<commit_message>
chore: update excel templates for autoclave and steri-vac
</commit_message>
<xml_diff>
--- a/public/templates/MANTTO PREVENTIVO DE STERI-VAC OE-01.xlsx
+++ b/public/templates/MANTTO PREVENTIVO DE STERI-VAC OE-01.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\emontes\Desktop\CONFORMIDAD AC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\willi\Desktop\MTTO.ASEPSIS.PE\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62B7A1AE-843E-4027-A506-6C2E3A19CFE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{24FFD954-65E3-4A7B-AD8E-CFAFEF32FE22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{22913600-765C-48AF-B40C-4C360125ED0D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{22913600-765C-48AF-B40C-4C360125ED0D}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Hoja1!$A$1:$P$32</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Hoja1!$A$1:$S$32</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -32,12 +32,15 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="52">
   <si>
     <t>Desmontaje y limpieza de linea de aire comprimido</t>
   </si>
@@ -180,30 +183,6 @@
     <t>Equipo queda operativo</t>
   </si>
   <si>
-    <t>LEYENDA:</t>
-  </si>
-  <si>
-    <t>(M) MENSUAL</t>
-  </si>
-  <si>
-    <t>(T) TRIMESTRAL</t>
-  </si>
-  <si>
-    <t>(S) SEMESTRAL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REALIZADO </t>
-  </si>
-  <si>
-    <t xml:space="preserve">APROBADO </t>
-  </si>
-  <si>
-    <t>(A) ANUAL</t>
-  </si>
-  <si>
-    <t>MANTENIMIENTO</t>
-  </si>
-  <si>
     <t>A</t>
   </si>
   <si>
@@ -211,6 +190,12 @@
   </si>
   <si>
     <t>Fecha: 02/2026</t>
+  </si>
+  <si>
+    <t>4XL - T</t>
+  </si>
+  <si>
+    <t>5XL -T</t>
   </si>
 </sst>
 </file>
@@ -242,12 +227,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="13">
@@ -394,7 +385,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -428,19 +419,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="4"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" indent="33"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -460,72 +458,102 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>160020</xdr:colOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>30480</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>45720</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>1485900</xdr:colOff>
+      <xdr:colOff>1478280</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>93588</xdr:rowOff>
+      <xdr:rowOff>144610</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Imagen 1" descr="Descripción: Imagen1">
+        <xdr:cNvPr id="3" name="Imagen 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4A8AB197-1C8A-42D5-BBBE-99C12FAA277B}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ED3E97BB-3C03-4F31-8460-85CCB9842119}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+          <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
         <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
           <a:extLst>
-            <a:ext uri="{BEBA8EAE-BF5A-486C-A8C5-ECC9F3942E4B}">
-              <a14:imgProps xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-                <a14:imgLayer r:embed="rId2">
-                  <a14:imgEffect>
-                    <a14:sharpenSoften amount="100000"/>
-                  </a14:imgEffect>
-                </a14:imgLayer>
-              </a14:imgProps>
-            </a:ext>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
             </a:ext>
           </a:extLst>
         </a:blip>
-        <a:srcRect/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
+      <xdr:spPr>
         <a:xfrm>
-          <a:off x="160020" y="45720"/>
-          <a:ext cx="1729740" cy="444108"/>
+          <a:off x="434340" y="0"/>
+          <a:ext cx="1447800" cy="540850"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>274321</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>91440</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>927033</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>147159</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Imagen 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7FC6A183-A0D4-457C-B7F8-4F1ED85E0A99}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8732521" y="3749040"/>
+          <a:ext cx="1864292" cy="1335879"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -830,19 +858,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDED3159-853A-4B06-AD7E-01BF4FB66868}">
-  <dimension ref="A1:P32"/>
+  <dimension ref="A1:T35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.88671875" customWidth="1"/>
     <col min="2" max="2" width="53.88671875" customWidth="1"/>
-    <col min="3" max="12" width="5.33203125" customWidth="1"/>
-    <col min="13" max="13" width="3.77734375" customWidth="1"/>
-    <col min="14" max="14" width="13.21875" customWidth="1"/>
-    <col min="15" max="15" width="4.44140625" customWidth="1"/>
-    <col min="16" max="16" width="16.6640625" customWidth="1"/>
+    <col min="3" max="11" width="5.33203125" customWidth="1"/>
+    <col min="12" max="12" width="6" customWidth="1"/>
+    <col min="13" max="13" width="6.44140625" customWidth="1"/>
+    <col min="14" max="14" width="6.5546875" customWidth="1"/>
+    <col min="15" max="15" width="5.33203125" customWidth="1"/>
+    <col min="16" max="16" width="3.77734375" customWidth="1"/>
+    <col min="17" max="17" width="13.21875" customWidth="1"/>
+    <col min="18" max="18" width="4.44140625" customWidth="1"/>
+    <col min="19" max="19" width="16.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="4"/>
       <c r="B1" s="14" t="s">
         <v>28</v>
@@ -859,22 +891,25 @@
       <c r="L1" s="5"/>
       <c r="M1" s="5"/>
       <c r="N1" s="5"/>
-      <c r="O1" s="6"/>
-      <c r="P1" s="2" t="s">
+      <c r="O1" s="5"/>
+      <c r="P1" s="5"/>
+      <c r="Q1" s="5"/>
+      <c r="R1" s="6"/>
+      <c r="S1" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:19" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="7"/>
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="O2" s="23"/>
-      <c r="P2" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="R2" s="20"/>
+      <c r="S2" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A3" s="8"/>
       <c r="B3" s="9"/>
       <c r="C3" s="9"/>
@@ -889,17 +924,20 @@
       <c r="L3" s="9"/>
       <c r="M3" s="9"/>
       <c r="N3" s="9"/>
-      <c r="O3" s="10"/>
-      <c r="P3" s="2" t="s">
+      <c r="O3" s="9"/>
+      <c r="P3" s="9"/>
+      <c r="Q3" s="9"/>
+      <c r="R3" s="10"/>
+      <c r="S3" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.3">
       <c r="K5" s="15"/>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>30</v>
@@ -931,10 +969,17 @@
       <c r="L6" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="M6" s="3"/>
-      <c r="N6" s="3"/>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="M6" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="N6" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="O6" s="3"/>
+      <c r="P6" s="3"/>
+      <c r="Q6" s="3"/>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>1</v>
       </c>
@@ -950,16 +995,19 @@
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
       <c r="K7" s="1" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="L7" s="2"/>
-      <c r="N7" s="16" t="s">
+      <c r="M7" s="2"/>
+      <c r="N7" s="2"/>
+      <c r="O7" s="21"/>
+      <c r="Q7" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="O7" s="17"/>
-      <c r="P7" s="13"/>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="R7" s="17"/>
+      <c r="S7" s="13"/>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>2</v>
       </c>
@@ -975,16 +1023,19 @@
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
       <c r="K8" s="1" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="L8" s="2"/>
-      <c r="N8" s="4" t="s">
+      <c r="M8" s="2"/>
+      <c r="N8" s="2"/>
+      <c r="O8" s="21"/>
+      <c r="Q8" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="O8" s="5"/>
-      <c r="P8" s="6"/>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="R8" s="5"/>
+      <c r="S8" s="6"/>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>3</v>
       </c>
@@ -1000,16 +1051,19 @@
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
       <c r="K9" s="1" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="L9" s="2"/>
-      <c r="N9" s="11" t="s">
+      <c r="M9" s="2"/>
+      <c r="N9" s="2"/>
+      <c r="O9" s="21"/>
+      <c r="Q9" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="O9" s="12"/>
-      <c r="P9" s="13"/>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="R9" s="12"/>
+      <c r="S9" s="13"/>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>4</v>
       </c>
@@ -1025,16 +1079,19 @@
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
       <c r="K10" s="1" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="L10" s="2"/>
-      <c r="N10" s="11" t="s">
+      <c r="M10" s="2"/>
+      <c r="N10" s="2"/>
+      <c r="O10" s="21"/>
+      <c r="Q10" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="O10" s="12"/>
-      <c r="P10" s="13"/>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="R10" s="12"/>
+      <c r="S10" s="13"/>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>5</v>
       </c>
@@ -1050,16 +1107,19 @@
       <c r="I11" s="1"/>
       <c r="J11" s="1"/>
       <c r="K11" s="1" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="L11" s="2"/>
-      <c r="N11" s="8" t="s">
+      <c r="M11" s="2"/>
+      <c r="N11" s="2"/>
+      <c r="O11" s="21"/>
+      <c r="Q11" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="O11" s="9"/>
-      <c r="P11" s="10"/>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="R11" s="9"/>
+      <c r="S11" s="10"/>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>6</v>
       </c>
@@ -1075,11 +1135,14 @@
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>
       <c r="K12" s="1" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="L12" s="2"/>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="M12" s="2"/>
+      <c r="N12" s="2"/>
+      <c r="O12" s="21"/>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>7</v>
       </c>
@@ -1095,11 +1158,19 @@
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>
       <c r="K13" s="1" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="L13" s="2"/>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="M13" s="2"/>
+      <c r="N13" s="2"/>
+      <c r="O13" s="21"/>
+      <c r="Q13" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="R13" s="12"/>
+      <c r="S13" s="13"/>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>8</v>
       </c>
@@ -1115,11 +1186,19 @@
       <c r="I14" s="1"/>
       <c r="J14" s="1"/>
       <c r="K14" s="1" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="L14" s="2"/>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="M14" s="2"/>
+      <c r="N14" s="2"/>
+      <c r="O14" s="21"/>
+      <c r="Q14" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="R14" s="5"/>
+      <c r="S14" s="6"/>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>9</v>
       </c>
@@ -1135,16 +1214,19 @@
       <c r="I15" s="1"/>
       <c r="J15" s="1"/>
       <c r="K15" s="1" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="L15" s="2"/>
-      <c r="N15" s="18" t="s">
-        <v>40</v>
-      </c>
-      <c r="O15" s="12"/>
-      <c r="P15" s="13"/>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="M15" s="2"/>
+      <c r="N15" s="2"/>
+      <c r="O15" s="21"/>
+      <c r="Q15" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="R15" s="12"/>
+      <c r="S15" s="13"/>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>10</v>
       </c>
@@ -1160,16 +1242,14 @@
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
       <c r="K16" s="1" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="L16" s="2"/>
-      <c r="N16" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="O16" s="5"/>
-      <c r="P16" s="6"/>
-    </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="M16" s="2"/>
+      <c r="N16" s="2"/>
+      <c r="O16" s="21"/>
+    </row>
+    <row r="17" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>11</v>
       </c>
@@ -1185,16 +1265,19 @@
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
       <c r="K17" s="1" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="L17" s="2"/>
-      <c r="N17" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="O17" s="12"/>
-      <c r="P17" s="13"/>
-    </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="M17" s="2"/>
+      <c r="N17" s="2"/>
+      <c r="O17" s="21"/>
+      <c r="Q17" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="R17" s="12"/>
+      <c r="S17" s="13"/>
+    </row>
+    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>12</v>
       </c>
@@ -1210,11 +1293,19 @@
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
       <c r="K18" s="1" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="L18" s="2"/>
-    </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="M18" s="2"/>
+      <c r="N18" s="2"/>
+      <c r="O18" s="21"/>
+      <c r="Q18" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="R18" s="5"/>
+      <c r="S18" s="6"/>
+    </row>
+    <row r="19" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>13</v>
       </c>
@@ -1230,11 +1321,19 @@
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
       <c r="K19" s="1" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="L19" s="2"/>
-    </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="M19" s="2"/>
+      <c r="N19" s="2"/>
+      <c r="O19" s="21"/>
+      <c r="Q19" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="R19" s="12"/>
+      <c r="S19" s="13"/>
+    </row>
+    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>14</v>
       </c>
@@ -1250,11 +1349,19 @@
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
       <c r="K20" s="1" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="L20" s="2"/>
-    </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="M20" s="2"/>
+      <c r="N20" s="2"/>
+      <c r="O20" s="21"/>
+      <c r="Q20" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="R20" s="9"/>
+      <c r="S20" s="10"/>
+    </row>
+    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>15</v>
       </c>
@@ -1270,16 +1377,14 @@
       <c r="I21" s="1"/>
       <c r="J21" s="1"/>
       <c r="K21" s="1" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="L21" s="2"/>
-      <c r="N21" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="O21" s="12"/>
-      <c r="P21" s="13"/>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="M21" s="2"/>
+      <c r="N21" s="2"/>
+      <c r="O21" s="21"/>
+    </row>
+    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>16</v>
       </c>
@@ -1295,17 +1400,20 @@
       <c r="I22" s="1"/>
       <c r="J22" s="1"/>
       <c r="K22" s="1" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="L22" s="2"/>
-      <c r="N22" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="O22" s="5"/>
-      <c r="P22" s="6"/>
-    </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A23" s="1"/>
+      <c r="M22" s="2"/>
+      <c r="N22" s="2"/>
+      <c r="O22" s="21"/>
+      <c r="Q22" s="24"/>
+      <c r="R22" s="25"/>
+      <c r="S22" s="26"/>
+    </row>
+    <row r="23" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A23" s="1">
+        <v>17</v>
+      </c>
       <c r="B23" s="2" t="s">
         <v>16</v>
       </c>
@@ -1318,16 +1426,17 @@
       <c r="I23" s="1"/>
       <c r="J23" s="1"/>
       <c r="K23" s="1" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="L23" s="2"/>
-      <c r="N23" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="O23" s="12"/>
-      <c r="P23" s="13"/>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="M23" s="2"/>
+      <c r="N23" s="2"/>
+      <c r="O23" s="21"/>
+      <c r="Q23" s="27"/>
+      <c r="R23" s="28"/>
+      <c r="S23" s="29"/>
+    </row>
+    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>18</v>
       </c>
@@ -1343,16 +1452,17 @@
       <c r="I24" s="1"/>
       <c r="J24" s="1"/>
       <c r="K24" s="1" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="L24" s="2"/>
-      <c r="N24" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="O24" s="9"/>
-      <c r="P24" s="10"/>
-    </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="M24" s="2"/>
+      <c r="N24" s="2"/>
+      <c r="O24" s="21"/>
+      <c r="Q24" s="27"/>
+      <c r="R24" s="28"/>
+      <c r="S24" s="29"/>
+    </row>
+    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>19</v>
       </c>
@@ -1368,11 +1478,17 @@
       <c r="I25" s="1"/>
       <c r="J25" s="1"/>
       <c r="K25" s="1" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="L25" s="2"/>
-    </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="M25" s="2"/>
+      <c r="N25" s="2"/>
+      <c r="O25" s="21"/>
+      <c r="Q25" s="27"/>
+      <c r="R25" s="28"/>
+      <c r="S25" s="29"/>
+    </row>
+    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
         <v>20</v>
       </c>
@@ -1388,11 +1504,17 @@
       <c r="I26" s="1"/>
       <c r="J26" s="1"/>
       <c r="K26" s="1" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="L26" s="2"/>
-    </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="M26" s="2"/>
+      <c r="N26" s="2"/>
+      <c r="O26" s="21"/>
+      <c r="Q26" s="27"/>
+      <c r="R26" s="28"/>
+      <c r="S26" s="29"/>
+    </row>
+    <row r="27" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
         <v>21</v>
       </c>
@@ -1408,41 +1530,139 @@
       <c r="I27" s="1"/>
       <c r="J27" s="1"/>
       <c r="K27" s="1" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="L27" s="2"/>
-    </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="G29" t="s">
-        <v>47</v>
-      </c>
-      <c r="I29" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="I30" s="19" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="I31" t="s">
-        <v>50</v>
-      </c>
-      <c r="N31" s="20" t="s">
-        <v>51</v>
-      </c>
-      <c r="P31" s="20" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="I32" t="s">
-        <v>53</v>
-      </c>
-      <c r="P32" s="21" t="s">
-        <v>54</v>
-      </c>
+      <c r="M27" s="2"/>
+      <c r="N27" s="2"/>
+      <c r="O27" s="21"/>
+      <c r="Q27" s="27"/>
+      <c r="R27" s="28"/>
+      <c r="S27" s="29"/>
+    </row>
+    <row r="28" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="Q28" s="27"/>
+      <c r="R28" s="28"/>
+      <c r="S28" s="29"/>
+    </row>
+    <row r="29" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="F29" s="21"/>
+      <c r="G29" s="21"/>
+      <c r="H29" s="21"/>
+      <c r="I29" s="21"/>
+      <c r="J29" s="21"/>
+      <c r="K29" s="21"/>
+      <c r="L29" s="21"/>
+      <c r="M29" s="21"/>
+      <c r="N29" s="21"/>
+      <c r="O29" s="21"/>
+      <c r="P29" s="21"/>
+      <c r="Q29" s="30"/>
+      <c r="R29" s="31"/>
+      <c r="S29" s="32"/>
+      <c r="T29" s="21"/>
+    </row>
+    <row r="30" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="F30" s="21"/>
+      <c r="G30" s="21"/>
+      <c r="H30" s="21"/>
+      <c r="I30" s="22"/>
+      <c r="J30" s="21"/>
+      <c r="K30" s="21"/>
+      <c r="L30" s="21"/>
+      <c r="M30" s="21"/>
+      <c r="N30" s="21"/>
+      <c r="O30" s="21"/>
+      <c r="P30" s="21"/>
+      <c r="Q30" s="21"/>
+      <c r="R30" s="21"/>
+      <c r="S30" s="21"/>
+      <c r="T30" s="21"/>
+    </row>
+    <row r="31" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="F31" s="21"/>
+      <c r="G31" s="21"/>
+      <c r="H31" s="21"/>
+      <c r="I31" s="21"/>
+      <c r="J31" s="21"/>
+      <c r="K31" s="21"/>
+      <c r="L31" s="21"/>
+      <c r="M31" s="21"/>
+      <c r="N31" s="21"/>
+      <c r="O31" s="21"/>
+      <c r="P31" s="21"/>
+      <c r="Q31" s="23"/>
+      <c r="R31" s="21"/>
+      <c r="S31" s="23"/>
+      <c r="T31" s="21"/>
+    </row>
+    <row r="32" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="F32" s="21"/>
+      <c r="G32" s="21"/>
+      <c r="H32" s="21"/>
+      <c r="I32" s="21"/>
+      <c r="J32" s="21"/>
+      <c r="K32" s="21"/>
+      <c r="L32" s="21"/>
+      <c r="M32" s="21"/>
+      <c r="N32" s="21"/>
+      <c r="O32" s="21"/>
+      <c r="P32" s="21"/>
+      <c r="Q32" s="21"/>
+      <c r="R32" s="21"/>
+      <c r="S32" s="23"/>
+      <c r="T32" s="21"/>
+    </row>
+    <row r="33" spans="6:20" x14ac:dyDescent="0.3">
+      <c r="F33" s="21"/>
+      <c r="G33" s="21"/>
+      <c r="H33" s="21"/>
+      <c r="I33" s="21"/>
+      <c r="J33" s="21"/>
+      <c r="K33" s="21"/>
+      <c r="L33" s="21"/>
+      <c r="M33" s="21"/>
+      <c r="N33" s="21"/>
+      <c r="O33" s="21"/>
+      <c r="P33" s="21"/>
+      <c r="Q33" s="21"/>
+      <c r="R33" s="21"/>
+      <c r="S33" s="21"/>
+      <c r="T33" s="21"/>
+    </row>
+    <row r="34" spans="6:20" x14ac:dyDescent="0.3">
+      <c r="F34" s="21"/>
+      <c r="G34" s="21"/>
+      <c r="H34" s="21"/>
+      <c r="I34" s="21"/>
+      <c r="J34" s="21"/>
+      <c r="K34" s="21"/>
+      <c r="L34" s="21"/>
+      <c r="M34" s="21"/>
+      <c r="N34" s="21"/>
+      <c r="O34" s="21"/>
+      <c r="P34" s="21"/>
+      <c r="Q34" s="21"/>
+      <c r="R34" s="21"/>
+      <c r="S34" s="21"/>
+      <c r="T34" s="21"/>
+    </row>
+    <row r="35" spans="6:20" x14ac:dyDescent="0.3">
+      <c r="F35" s="21"/>
+      <c r="G35" s="21"/>
+      <c r="H35" s="21"/>
+      <c r="I35" s="21"/>
+      <c r="J35" s="21"/>
+      <c r="K35" s="21"/>
+      <c r="L35" s="21"/>
+      <c r="M35" s="21"/>
+      <c r="N35" s="21"/>
+      <c r="O35" s="21"/>
+      <c r="P35" s="21"/>
+      <c r="Q35" s="21"/>
+      <c r="R35" s="21"/>
+      <c r="S35" s="21"/>
+      <c r="T35" s="21"/>
     </row>
   </sheetData>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>